<commit_message>
solved ciphers 1 & 3, 2 started
</commit_message>
<xml_diff>
--- a/cw/docs/cipher-notes.xlsx
+++ b/cw/docs/cipher-notes.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deric\OneDrive\Desktop\School\Year_4\Semester_2\Cryptography\cw\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA78B38A-13C6-415C-A952-6457CC442EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB27973-C2EC-456F-B4D2-7E8E930D016A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51705" yWindow="-5160" windowWidth="26010" windowHeight="20985" xr2:uid="{138468FD-49EB-489D-ABA2-5E2D296F7952}"/>
+    <workbookView xWindow="-51705" yWindow="-5160" windowWidth="15285" windowHeight="20985" xr2:uid="{138468FD-49EB-489D-ABA2-5E2D296F7952}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Cipher 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Cipher 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Cipher 3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,11 +38,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="43">
   <si>
     <t>A</t>
   </si>
   <si>
+    <t>B</t>
+  </si>
+  <si>
     <t>C</t>
   </si>
   <si>
@@ -68,6 +73,12 @@
     <t>Substitution</t>
   </si>
   <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
     <t>U</t>
   </si>
   <si>
@@ -83,6 +94,9 @@
     <t>I</t>
   </si>
   <si>
+    <t>L</t>
+  </si>
+  <si>
     <t>V</t>
   </si>
   <si>
@@ -93,6 +107,66 @@
   </si>
   <si>
     <t>J</t>
+  </si>
+  <si>
+    <t>Factors of 66:</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>e</t>
+  </si>
+  <si>
+    <t>o</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>l</t>
+  </si>
+  <si>
+    <t>u</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>t</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>w</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>N</t>
   </si>
 </sst>
 </file>
@@ -496,7 +570,7 @@
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -604,67 +678,805 @@
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
+        <v>10</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="I2" s="3" t="s">
+      <c r="K2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="W2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="J2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="S2" s="3" t="s">
+      <c r="X2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="T2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="W2" s="3" t="s">
+      <c r="Y2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="X2" s="3" t="s">
+      <c r="Z2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="Y2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="Z2" s="3"/>
       <c r="AA2" s="3" t="s">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F620D8A-BA8D-4A5C-92A7-8A9FADA1EF8E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29A94DB3-7B8A-455C-9533-DF977D964323}">
+  <dimension ref="A1:G38"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="2.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="2.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="2.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="2.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="2.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="2.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="1">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1">
+        <v>66</v>
+      </c>
+      <c r="C2" s="1">
+        <v>33</v>
+      </c>
+      <c r="D2" s="1">
+        <v>22</v>
+      </c>
+      <c r="E2" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B16" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B17" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B20" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B21" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B22" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B23" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B24" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B25" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B26" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B28" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B29" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B30" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B31" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B32" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B33" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B34" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B35" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B36" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B37" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B38" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>